<commit_message>
Generate July 2026 report with June data from updated operating record.
Refresh June plots, operations schedule table, and LaTeX narrative using the latest WA25001 Excel log with expanded mid- and late-June WETA activity.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/raw/WA25001_Flat_Iron_UT_HVG_Operating_Record_v01.xlsx
+++ b/data/raw/WA25001_Flat_Iron_UT_HVG_Operating_Record_v01.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="13">
   <si>
     <t>WA25001 Operating Times</t>
   </si>
@@ -2306,11 +2306,21 @@
       <c r="Z51" s="6"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="6"/>
-      <c r="B52" s="6"/>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
+      <c r="A52" s="12">
+        <v>46185.0</v>
+      </c>
+      <c r="B52" s="9">
+        <v>926.0</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D52" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E52" s="9">
+        <v>0.0</v>
+      </c>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
       <c r="H52" s="6"/>
@@ -2334,11 +2344,21 @@
       <c r="Z52" s="6"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="6"/>
-      <c r="B53" s="6"/>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
-      <c r="E53" s="6"/>
+      <c r="A53" s="12">
+        <v>46189.0</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" s="9">
+        <v>636.0</v>
+      </c>
+      <c r="D53" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E53" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F53" s="6"/>
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
@@ -2362,11 +2382,21 @@
       <c r="Z53" s="6"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="6"/>
-      <c r="B54" s="6"/>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6"/>
+      <c r="A54" s="12">
+        <v>46196.0</v>
+      </c>
+      <c r="B54" s="9">
+        <v>549.0</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E54" s="9">
+        <v>0.0</v>
+      </c>
       <c r="F54" s="6"/>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
@@ -2390,11 +2420,21 @@
       <c r="Z54" s="6"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="6"/>
-      <c r="B55" s="6"/>
-      <c r="C55" s="6"/>
-      <c r="D55" s="6"/>
-      <c r="E55" s="6"/>
+      <c r="A55" s="12">
+        <v>46202.0</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C55" s="9">
+        <v>1226.0</v>
+      </c>
+      <c r="D55" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E55" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F55" s="6"/>
       <c r="G55" s="6"/>
       <c r="H55" s="6"/>
@@ -2418,11 +2458,21 @@
       <c r="Z55" s="6"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="6"/>
-      <c r="B56" s="6"/>
-      <c r="C56" s="6"/>
-      <c r="D56" s="6"/>
-      <c r="E56" s="6"/>
+      <c r="A56" s="12">
+        <v>46209.0</v>
+      </c>
+      <c r="B56" s="9">
+        <v>1107.0</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E56" s="9">
+        <v>0.0</v>
+      </c>
       <c r="F56" s="6"/>
       <c r="G56" s="6"/>
       <c r="H56" s="6"/>

</xml_diff>

<commit_message>
Update August report with July 2026 operations and warm-season analysis.
Align main.tex with the revised PDF structure, refresh WETA schedule from the operating record, use Buckboard Flat as the Gold Basin control, and add July plots plus analog-year enhancement estimates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/raw/WA25001_Flat_Iron_UT_HVG_Operating_Record_v01.xlsx
+++ b/data/raw/WA25001_Flat_Iron_UT_HVG_Operating_Record_v01.xlsx
@@ -11,14 +11,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="CRZSGqi366Vc7aUcyBI8vf1m7/ZUxsb5cPL/OT9d+LU="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="GuPrjYLV+qRMpUIRRzrgAkQV+FzRYJ+jlGMzyd8VD+s="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="14">
   <si>
     <t>WA25001 Operating Times</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>Dry start...</t>
+  </si>
+  <si>
+    <t>Dry start</t>
   </si>
 </sst>
 </file>
@@ -2496,11 +2499,21 @@
       <c r="Z56" s="6"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="6"/>
-      <c r="B57" s="6"/>
-      <c r="C57" s="6"/>
-      <c r="D57" s="6"/>
-      <c r="E57" s="6"/>
+      <c r="A57" s="12">
+        <v>46212.0</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C57" s="9">
+        <v>1359.0</v>
+      </c>
+      <c r="D57" s="9">
+        <v>99.8</v>
+      </c>
+      <c r="E57" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F57" s="6"/>
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
@@ -2524,11 +2537,21 @@
       <c r="Z57" s="6"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="6"/>
-      <c r="B58" s="6"/>
-      <c r="C58" s="6"/>
-      <c r="D58" s="6"/>
-      <c r="E58" s="6"/>
+      <c r="A58" s="12">
+        <v>46214.0</v>
+      </c>
+      <c r="B58" s="9">
+        <v>1813.0</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E58" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F58" s="6"/>
       <c r="G58" s="6"/>
       <c r="H58" s="6"/>
@@ -2552,11 +2575,21 @@
       <c r="Z58" s="6"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="6"/>
-      <c r="B59" s="6"/>
-      <c r="C59" s="6"/>
-      <c r="D59" s="6"/>
-      <c r="E59" s="6"/>
+      <c r="A59" s="12">
+        <v>46224.0</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C59" s="9">
+        <v>1213.0</v>
+      </c>
+      <c r="D59" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E59" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F59" s="6"/>
       <c r="G59" s="6"/>
       <c r="H59" s="6"/>
@@ -2580,11 +2613,21 @@
       <c r="Z59" s="6"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="6"/>
-      <c r="B60" s="6"/>
-      <c r="C60" s="6"/>
-      <c r="D60" s="6"/>
-      <c r="E60" s="6"/>
+      <c r="A60" s="12">
+        <v>46225.0</v>
+      </c>
+      <c r="B60" s="9">
+        <v>455.0</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E60" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F60" s="6"/>
       <c r="G60" s="6"/>
       <c r="H60" s="6"/>
@@ -2608,11 +2651,21 @@
       <c r="Z60" s="6"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="6"/>
-      <c r="B61" s="6"/>
-      <c r="C61" s="6"/>
-      <c r="D61" s="6"/>
-      <c r="E61" s="6"/>
+      <c r="A61" s="12">
+        <v>46225.0</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C61" s="9">
+        <v>1231.0</v>
+      </c>
+      <c r="D61" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E61" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F61" s="6"/>
       <c r="G61" s="6"/>
       <c r="H61" s="6"/>
@@ -2636,11 +2689,21 @@
       <c r="Z61" s="6"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="6"/>
-      <c r="B62" s="6"/>
-      <c r="C62" s="6"/>
-      <c r="D62" s="6"/>
-      <c r="E62" s="6"/>
+      <c r="A62" s="12">
+        <v>46227.0</v>
+      </c>
+      <c r="B62" s="9">
+        <v>2113.0</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E62" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F62" s="6"/>
       <c r="G62" s="6"/>
       <c r="H62" s="6"/>
@@ -2664,11 +2727,21 @@
       <c r="Z62" s="6"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="6"/>
-      <c r="B63" s="6"/>
-      <c r="C63" s="6"/>
-      <c r="D63" s="6"/>
-      <c r="E63" s="6"/>
+      <c r="A63" s="12">
+        <v>46237.0</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C63" s="9">
+        <v>1020.0</v>
+      </c>
+      <c r="D63" s="9">
+        <v>99.8</v>
+      </c>
+      <c r="E63" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F63" s="6"/>
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
@@ -2692,12 +2765,24 @@
       <c r="Z63" s="6"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="6"/>
-      <c r="B64" s="6"/>
-      <c r="C64" s="6"/>
-      <c r="D64" s="6"/>
-      <c r="E64" s="6"/>
-      <c r="F64" s="6"/>
+      <c r="A64" s="12">
+        <v>46241.0</v>
+      </c>
+      <c r="B64" s="9">
+        <v>630.0</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E64" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="F64" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
       <c r="I64" s="6"/>
@@ -2720,11 +2805,21 @@
       <c r="Z64" s="6"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="6"/>
-      <c r="B65" s="6"/>
-      <c r="C65" s="6"/>
-      <c r="D65" s="6"/>
-      <c r="E65" s="6"/>
+      <c r="A65" s="13">
+        <v>46248.0</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C65" s="9">
+        <v>1307.0</v>
+      </c>
+      <c r="D65" s="9">
+        <v>99.8</v>
+      </c>
+      <c r="E65" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F65" s="6"/>
       <c r="G65" s="6"/>
       <c r="H65" s="6"/>
@@ -2748,11 +2843,21 @@
       <c r="Z65" s="6"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="6"/>
-      <c r="B66" s="6"/>
-      <c r="C66" s="6"/>
-      <c r="D66" s="6"/>
-      <c r="E66" s="6"/>
+      <c r="A66" s="12">
+        <v>46252.0</v>
+      </c>
+      <c r="B66" s="9">
+        <v>2012.0</v>
+      </c>
+      <c r="C66" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E66" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F66" s="6"/>
       <c r="G66" s="6"/>
       <c r="H66" s="6"/>
@@ -28955,34 +29060,6 @@
       <c r="Y1001" s="6"/>
       <c r="Z1001" s="6"/>
     </row>
-    <row r="1002" ht="15.75" customHeight="1">
-      <c r="A1002" s="6"/>
-      <c r="B1002" s="6"/>
-      <c r="C1002" s="6"/>
-      <c r="D1002" s="6"/>
-      <c r="E1002" s="6"/>
-      <c r="F1002" s="6"/>
-      <c r="G1002" s="6"/>
-      <c r="H1002" s="6"/>
-      <c r="I1002" s="6"/>
-      <c r="J1002" s="6"/>
-      <c r="K1002" s="6"/>
-      <c r="L1002" s="6"/>
-      <c r="M1002" s="6"/>
-      <c r="N1002" s="6"/>
-      <c r="O1002" s="6"/>
-      <c r="P1002" s="6"/>
-      <c r="Q1002" s="6"/>
-      <c r="R1002" s="6"/>
-      <c r="S1002" s="6"/>
-      <c r="T1002" s="6"/>
-      <c r="U1002" s="6"/>
-      <c r="V1002" s="6"/>
-      <c r="W1002" s="6"/>
-      <c r="X1002" s="6"/>
-      <c r="Y1002" s="6"/>
-      <c r="Z1002" s="6"/>
-    </row>
   </sheetData>
   <autoFilter ref="$A$2:$F$36"/>
   <mergeCells count="1">

</xml_diff>